<commit_message>
update: 2026/06/25 周四  9:05:01.48
</commit_message>
<xml_diff>
--- a/source/9、人数基数/人数基数-5月.xlsx
+++ b/source/9、人数基数/人数基数-5月.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="22400" windowHeight="10200"/>
+    <workbookView windowWidth="21550" windowHeight="10200"/>
   </bookViews>
   <sheets>
     <sheet name="人数基数模板" sheetId="1" r:id="rId1"/>
@@ -2445,7 +2445,7 @@
         <v>74</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>67</v>
+        <v>7</v>
       </c>
       <c r="D68" s="2">
         <v>288</v>

</xml_diff>